<commit_message>
fix: recalculate cart prices after pricelist reload
Accept persisted boolean service statuses during cart recalculation, in addition to Tkinter variable objects. This prevents the confirmation action after a pricelist reload from failing with AttributeError. Recalculate tool, coating, and additional service totals for existing cart items after the user confirms the new prices. Add regression coverage for saved boolean statuses and full cart item price recalculation.
</commit_message>
<xml_diff>
--- a/data/cennik.xlsx
+++ b/data/cennik.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Repository\Ostrzomat\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F7A31C-534E-442B-807D-D30980F3116A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D28AFF-F1CF-4A78-AC10-F99E5D17D9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2415" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -614,7 +614,7 @@
         <v>12</v>
       </c>
       <c r="G4">
-        <v>62.4</v>
+        <v>64.5</v>
       </c>
       <c r="H4">
         <v>49.1</v>

</xml_diff>